<commit_message>
Questionnaire de paramétrage AxisPro, mise en page commune avec celui de la finance
25 questions pour la direction et les consultants de MB AxisPro : grille et méthode
(seuils, pondération, validité des pièces), dossiers en cours, comités, modèle
financier, portail, temps et honoraires, autres activités du cabinet, utilisateurs.
Mise en page partagée (questionnaire_commun.py) ; « MB AxisPro » dans les textes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/projet/Questionnaire_parametrage_finance.xlsx
+++ b/docs/projet/Questionnaire_parametrage_finance.xlsx
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,7 +106,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -479,7 +478,7 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
@@ -494,7 +493,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>EGUITRA GROUP SARLU et MB AxisPro Consulting · plateforme NIMOVA</t>
+          <t>EGUITRA GROUP SARLU et MB AxisPro · plateforme NIMOVA</t>
         </is>
       </c>
     </row>
@@ -570,7 +569,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>MB AxisPro Consulting a-t-elle son propre classeur, ou ses opérations sont-elles dans celui d'EGUITRA GROUP ?</t>
+          <t>MB AxisPro a-t-elle son propre classeur, ou ses opérations sont-elles dans celui d'EGUITRA GROUP ?</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -727,7 +726,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Quel est le régime fiscal de chaque société, et les deux sont-elles assujetties à la TVA ? Quand a commencé le premier exercice de MB AxisPro Consulting ?</t>
+          <t>Quel est le régime fiscal de chaque société, et les deux sont-elles assujetties à la TVA ? Quand a commencé le premier exercice de MB AxisPro ?</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -1373,7 +1372,7 @@
   <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1386,255 +1385,255 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Pièce</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Remise le</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Classeur définitif</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="10" t="inlineStr"/>
+      <c r="C4" s="10" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Ces fichiers</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="10" t="inlineStr"/>
+      <c r="C5" s="10" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>États financiers 2025</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="10" t="inlineStr"/>
+      <c r="C6" s="10" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Contrats et échéanciers</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="10" t="inlineStr"/>
+      <c r="C7" s="10" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>RCCM, attestations NIF</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="10" t="inlineStr"/>
+      <c r="C8" s="10" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Soldes au 31/12/2025</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Liste des comptes utilisés</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="10" t="inlineStr"/>
+      <c r="C10" s="10" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Attestations d'exonération</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr"/>
+      <c r="C11" s="10" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Dernières déclarations</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="9" t="n">
         <v>19</v>
       </c>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr"/>
+      <c r="C12" s="10" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Une facture récente</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="10" t="inlineStr"/>
+      <c r="C13" s="10" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Grille tarifaire 2026</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="9" t="n">
         <v>22</v>
       </c>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="10" t="inlineStr"/>
+      <c r="C14" s="10" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Un exemple de chaque</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="9" t="n">
         <v>23</v>
       </c>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>RIB et soldes au 31/12/2025</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="C16" s="11" t="inlineStr"/>
-      <c r="D16" s="10" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Un relevé par banque</t>
         </is>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="9" t="n">
         <v>29</v>
       </c>
-      <c r="C17" s="11" t="inlineStr"/>
-      <c r="D17" s="10" t="inlineStr"/>
+      <c r="C17" s="10" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>Tableau des immobilisations</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="C18" s="11" t="inlineStr"/>
-      <c r="D18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>Liste des impayés</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="9" t="n">
         <v>32</v>
       </c>
-      <c r="C19" s="11" t="inlineStr"/>
-      <c r="D19" s="10" t="inlineStr"/>
+      <c r="C19" s="10" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>Budget 2026</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="9" t="n">
         <v>34</v>
       </c>
-      <c r="C20" s="11" t="inlineStr"/>
-      <c r="D20" s="10" t="inlineStr"/>
+      <c r="C20" s="10" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>Journal de paie d'un mois</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="9" t="n">
         <v>36</v>
       </c>
-      <c r="C21" s="11" t="inlineStr"/>
-      <c r="D21" s="10" t="inlineStr"/>
+      <c r="C21" s="10" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Liste nominative</t>
         </is>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="9" t="n">
         <v>37</v>
       </c>
-      <c r="C22" s="11" t="inlineStr"/>
-      <c r="D22" s="10" t="inlineStr"/>
+      <c r="C22" s="10" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>